<commit_message>
Update Quotation_Tracker.xlsx with demo entries
</commit_message>
<xml_diff>
--- a/Quotation_Tracker.xlsx
+++ b/Quotation_Tracker.xlsx
@@ -508,7 +508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -865,6 +865,230 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Rajby Industries</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>procurement@rajby.com</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>PR-2026-101</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Safety Gloves Heavy Duty</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Pairs</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>500</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr"/>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>19-Jun-2026</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>02:55 PM</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr"/>
+      <c r="M7" s="4" t="inlineStr"/>
+      <c r="N7" s="4" t="inlineStr"/>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Hunar Foundation</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>admin@hunar.org</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>PR-HF-045</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>A4 Paper 80 GSM</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Reams</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>850</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>19-Jun-2026</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>02:55 PM</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Rajby Industries</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>procurement@rajby.com</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>PR-2026-101</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Safety Helmets Yellow</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Nos</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr"/>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>19-Jun-2026</t>
+        </is>
+      </c>
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>02:55 PM</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr"/>
+      <c r="M9" s="4" t="inlineStr"/>
+      <c r="N9" s="4" t="inlineStr"/>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Al-Karam Textile</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>purchase@alkaram.com</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>PR-AK-009</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Industrial Lubricant Oil</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Ltrs</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>19-Jun-2026</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>02:55 PM</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>